<commit_message>
Normalize A1 levels and alternate Student A and Student B across all cards
</commit_message>
<xml_diff>
--- a/data/speakingcards_questions.xlsx
+++ b/data/speakingcards_questions.xlsx
@@ -507,7 +507,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -515,7 +515,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -539,7 +543,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -547,7 +551,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -571,7 +579,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -579,7 +587,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -603,7 +615,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -611,7 +623,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H5" s="2" t="n"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -635,7 +651,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -643,7 +659,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -667,7 +687,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -675,7 +695,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H7" s="2" t="n"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -699,7 +723,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -707,7 +731,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H8" s="2" t="n"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -731,7 +759,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -739,7 +767,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H9" s="2" t="n"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -763,7 +795,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -771,7 +803,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H10" s="2" t="n"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -795,7 +831,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -803,7 +839,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H11" s="2" t="n"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -827,7 +867,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -835,7 +875,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H12" s="2" t="n"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -859,7 +903,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -867,7 +911,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H13" s="2" t="n"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -891,7 +939,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -899,7 +947,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H14" s="2" t="n"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -923,7 +975,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -931,7 +983,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -955,7 +1011,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -963,7 +1019,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H16" s="2" t="n"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -987,7 +1047,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -995,7 +1055,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H17" s="2" t="n"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1019,7 +1083,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1027,7 +1091,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1051,7 +1119,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1059,7 +1127,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H19" s="2" t="n"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1083,7 +1155,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1091,7 +1163,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H20" s="2" t="n"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1115,7 +1191,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1123,7 +1199,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H21" s="2" t="n"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1147,7 +1227,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1155,7 +1235,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H22" s="2" t="n"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1183,7 +1267,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -1191,7 +1275,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H23" s="2" t="n"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1219,7 +1307,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1227,7 +1315,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1251,7 +1343,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -1259,7 +1351,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1283,7 +1379,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -1291,7 +1387,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H26" s="2" t="n"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1315,7 +1415,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -1323,7 +1423,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H27" s="2" t="n"/>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1347,7 +1451,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -1355,7 +1459,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H28" s="2" t="n"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1383,7 +1491,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1391,7 +1499,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H29" s="2" t="n"/>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1419,7 +1531,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -1427,7 +1539,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H30" s="2" t="n"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1451,7 +1567,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -1459,7 +1575,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H31" s="2" t="n"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1483,7 +1603,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -1491,7 +1611,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1519,7 +1643,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -1527,7 +1651,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H33" s="2" t="n"/>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1551,7 +1679,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1559,7 +1687,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1583,7 +1715,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -1591,7 +1723,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H35" s="2" t="n"/>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1615,7 +1751,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -1623,7 +1759,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H36" s="2" t="n"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1647,7 +1787,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -1655,7 +1795,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H37" s="2" t="n"/>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1679,7 +1823,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -1687,7 +1831,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H38" s="2" t="n"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1711,7 +1859,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -1719,7 +1867,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H39" s="2" t="n"/>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1743,7 +1895,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -1751,7 +1903,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H40" s="2" t="n"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1775,7 +1931,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -1783,7 +1939,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H41" s="2" t="n"/>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1807,7 +1967,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -1815,7 +1975,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H42" s="2" t="n"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1839,7 +2003,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -1847,7 +2011,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H43" s="2" t="n"/>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1871,7 +2039,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -1879,7 +2047,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H44" s="2" t="n"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1903,7 +2075,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -1911,7 +2083,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H45" s="2" t="n"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1935,7 +2111,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -1943,7 +2119,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H46" s="2" t="n"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1967,7 +2147,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -1975,7 +2155,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H47" s="2" t="n"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1999,7 +2183,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -2007,7 +2191,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H48" s="2" t="n"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2031,7 +2219,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -2039,7 +2227,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H49" s="2" t="n"/>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2063,7 +2255,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2071,7 +2263,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H50" s="2" t="n"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2099,7 +2295,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -2107,7 +2303,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H51" s="2" t="n"/>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2131,7 +2331,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -2139,7 +2339,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H52" s="2" t="n"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2163,7 +2367,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -2171,7 +2375,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H53" s="2" t="n"/>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2195,7 +2403,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -2203,7 +2411,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H54" s="2" t="n"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2227,7 +2439,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -2235,7 +2447,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H55" s="2" t="n"/>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2259,7 +2475,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -2267,7 +2483,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H56" s="2" t="n"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2291,7 +2511,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -2299,7 +2519,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H57" s="2" t="n"/>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2323,7 +2547,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -2331,7 +2555,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H58" s="2" t="n"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2355,7 +2583,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -2363,7 +2591,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H59" s="2" t="n"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2387,7 +2619,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -2395,7 +2627,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H60" s="2" t="n"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2419,7 +2655,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -2427,7 +2663,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H61" s="2" t="n"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2451,7 +2691,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -2459,7 +2699,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H62" s="2" t="n"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2483,7 +2727,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -2491,7 +2735,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H63" s="2" t="n"/>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2515,7 +2763,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -2523,7 +2771,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2547,7 +2799,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -2555,7 +2807,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H65" s="2" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2579,7 +2835,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -2587,7 +2843,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H66" s="2" t="n"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2611,7 +2871,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -2619,7 +2879,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H67" s="2" t="n"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2643,7 +2907,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -2651,7 +2915,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H68" s="2" t="n"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2675,7 +2943,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -2683,7 +2951,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2707,7 +2979,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -2715,7 +2987,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H70" s="2" t="n"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -2739,7 +3015,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -2747,7 +3023,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H71" s="2" t="n"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -2771,7 +3051,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -2779,7 +3059,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H72" s="2" t="n"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -2803,7 +3087,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -2811,7 +3095,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H73" s="2" t="n"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2835,7 +3123,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -2843,7 +3131,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H74" s="2" t="n"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -2867,7 +3159,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -2875,7 +3167,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H75" s="2" t="n"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2899,7 +3195,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -2907,7 +3203,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H76" s="2" t="n"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -2931,7 +3231,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -2939,7 +3239,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H77" s="2" t="n"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -2963,7 +3267,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -2971,7 +3275,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H78" s="2" t="n"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -2995,7 +3303,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -3003,7 +3311,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H79" s="2" t="n"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3027,7 +3339,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -3035,7 +3347,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H80" s="2" t="n"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3059,7 +3375,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -3067,7 +3383,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H81" s="2" t="n"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3091,7 +3411,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -3099,7 +3419,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H82" s="2" t="n"/>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3123,7 +3447,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -3131,7 +3455,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H83" s="2" t="n"/>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3155,7 +3483,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -3163,7 +3491,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H84" s="2" t="n"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3187,7 +3519,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -3195,7 +3527,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H85" s="2" t="n"/>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3219,7 +3555,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -3227,7 +3563,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H86" s="2" t="n"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3251,7 +3591,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -3259,7 +3599,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H87" s="2" t="n"/>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3283,7 +3627,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -3291,7 +3635,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H88" s="2" t="n"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3315,7 +3663,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -3323,7 +3671,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H89" s="2" t="n"/>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3347,7 +3699,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -3355,7 +3707,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H90" s="2" t="n"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3383,7 +3739,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -3391,7 +3747,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H91" s="2" t="n"/>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3415,7 +3775,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -3423,7 +3783,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H92" s="2" t="n"/>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3447,7 +3811,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -3455,7 +3819,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H93" s="2" t="n"/>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3479,7 +3847,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -3487,7 +3855,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H94" s="2" t="n"/>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3511,7 +3883,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -3519,7 +3891,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H95" s="2" t="n"/>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3543,7 +3919,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -3551,7 +3927,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H96" s="2" t="n"/>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3575,7 +3955,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -3583,7 +3963,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H97" s="2" t="n"/>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -3611,7 +3995,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -3619,7 +4003,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H98" s="2" t="n"/>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -3643,7 +4031,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -3651,7 +4039,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H99" s="2" t="n"/>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -3675,7 +4067,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -3683,7 +4075,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H100" s="2" t="n"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -3707,7 +4103,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -3715,7 +4111,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H101" s="2" t="n"/>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -3739,7 +4139,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -3747,7 +4147,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H102" s="2" t="n"/>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -3771,7 +4175,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -3779,7 +4183,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H103" s="2" t="n"/>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -3803,7 +4211,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -3811,7 +4219,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H104" s="2" t="n"/>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -3835,7 +4247,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -3843,7 +4255,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H105" s="2" t="n"/>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -3867,7 +4283,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -3875,7 +4291,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H106" s="2" t="n"/>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -3899,7 +4319,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -3907,7 +4327,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H107" s="2" t="n"/>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -3931,7 +4355,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -3939,7 +4363,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H108" s="2" t="n"/>
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -3963,7 +4391,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -3971,7 +4399,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H109" s="2" t="n"/>
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -3995,7 +4427,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -4003,7 +4435,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H110" s="2" t="n"/>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4027,7 +4463,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -4035,7 +4471,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H111" s="2" t="n"/>
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4059,7 +4499,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -4067,7 +4507,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H112" s="2" t="n"/>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4091,7 +4535,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -4099,7 +4543,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H113" s="2" t="n"/>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4123,7 +4571,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -4131,7 +4579,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H114" s="2" t="n"/>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4155,7 +4607,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -4163,7 +4615,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H115" s="2" t="n"/>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4187,7 +4643,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -4195,7 +4651,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H116" s="2" t="n"/>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4219,7 +4679,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -4227,7 +4687,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H117" s="2" t="n"/>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4251,7 +4715,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -4259,7 +4723,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H118" s="2" t="n"/>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4287,7 +4755,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -4295,7 +4763,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H119" s="2" t="n"/>
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4319,7 +4791,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -4327,7 +4799,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H120" s="2" t="n"/>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4351,7 +4827,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -4359,7 +4835,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H121" s="2" t="n"/>
+      <c r="H121" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4383,7 +4863,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -4391,7 +4871,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H122" s="2" t="n"/>
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4415,7 +4899,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -4423,7 +4907,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H123" s="2" t="n"/>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4447,7 +4935,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -4455,7 +4943,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H124" s="2" t="n"/>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4479,7 +4971,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -4487,7 +4979,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H125" s="2" t="n"/>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -4511,7 +5007,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -4519,7 +5015,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H126" s="2" t="n"/>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -4543,7 +5043,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -4551,7 +5051,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H127" s="2" t="n"/>
+      <c r="H127" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -4575,7 +5079,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -4583,7 +5087,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H128" s="2" t="n"/>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -4607,7 +5115,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -4615,7 +5123,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H129" s="2" t="n"/>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -4639,7 +5151,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -4647,7 +5159,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H130" s="2" t="n"/>
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -4671,7 +5187,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -4679,7 +5195,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H131" s="2" t="n"/>
+      <c r="H131" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -4703,7 +5223,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -4711,7 +5231,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H132" s="2" t="n"/>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -4735,7 +5259,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -4743,7 +5267,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H133" s="2" t="n"/>
+      <c r="H133" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -4767,7 +5295,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -4775,7 +5303,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H134" s="2" t="n"/>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -4799,7 +5331,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -4807,7 +5339,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H135" s="2" t="n"/>
+      <c r="H135" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -4831,7 +5367,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -4839,7 +5375,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H136" s="2" t="n"/>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -4863,7 +5403,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -4871,7 +5411,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H137" s="2" t="n"/>
+      <c r="H137" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -4895,7 +5439,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -4903,7 +5447,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H138" s="2" t="n"/>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -4927,7 +5475,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -4935,7 +5483,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H139" s="2" t="n"/>
+      <c r="H139" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -4959,7 +5511,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -4967,7 +5519,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H140" s="2" t="n"/>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -4991,7 +5547,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -4999,7 +5555,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H141" s="2" t="n"/>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5023,7 +5583,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -5031,7 +5591,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H142" s="2" t="n"/>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5055,7 +5619,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -5063,7 +5627,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H143" s="2" t="n"/>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5087,7 +5655,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -5095,7 +5663,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H144" s="2" t="n"/>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5119,7 +5691,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -5127,7 +5699,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H145" s="2" t="n"/>
+      <c r="H145" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5151,7 +5727,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -5159,7 +5735,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H146" s="2" t="n"/>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5183,7 +5763,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -5191,7 +5771,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H147" s="2" t="n"/>
+      <c r="H147" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5215,7 +5799,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -5223,7 +5807,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H148" s="2" t="n"/>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -5247,7 +5835,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -5255,7 +5843,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H149" s="2" t="n"/>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -5279,7 +5871,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -5287,7 +5879,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H150" s="2" t="n"/>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -5311,7 +5907,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -5319,7 +5915,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H151" s="2" t="n"/>
+      <c r="H151" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5343,7 +5943,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -5351,7 +5951,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H152" s="2" t="n"/>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5375,7 +5979,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -5383,7 +5987,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H153" s="2" t="n"/>
+      <c r="H153" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -5407,7 +6015,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -5415,7 +6023,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H154" s="2" t="n"/>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -5439,7 +6051,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -5447,7 +6059,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H155" s="2" t="n"/>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -5471,7 +6087,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -5479,7 +6095,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H156" s="2" t="n"/>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -5503,7 +6123,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -5511,7 +6131,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H157" s="2" t="n"/>
+      <c r="H157" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -5535,7 +6159,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -5543,7 +6167,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H158" s="2" t="n"/>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -5567,7 +6195,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -5575,7 +6203,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H159" s="2" t="n"/>
+      <c r="H159" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -5599,7 +6231,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -5607,7 +6239,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H160" s="2" t="n"/>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -5631,7 +6267,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -5639,7 +6275,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H161" s="2" t="n"/>
+      <c r="H161" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -5663,7 +6303,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -5671,7 +6311,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H162" s="2" t="n"/>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -5695,7 +6339,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -5703,7 +6347,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H163" s="2" t="n"/>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -5727,7 +6375,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -5735,7 +6383,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H164" s="2" t="n"/>
+      <c r="H164" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -5759,7 +6411,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -5767,7 +6419,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H165" s="2" t="n"/>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -5791,7 +6447,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -5799,7 +6455,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H166" s="2" t="n"/>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -5823,7 +6483,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -5831,7 +6491,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H167" s="2" t="n"/>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -5855,7 +6519,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -5863,7 +6527,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H168" s="2" t="n"/>
+      <c r="H168" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -5887,7 +6555,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -5895,7 +6563,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H169" s="2" t="n"/>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -5919,7 +6591,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -5927,7 +6599,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H170" s="2" t="n"/>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -5951,7 +6627,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>A1.1</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -5959,7 +6635,11 @@
           <t>A1.1</t>
         </is>
       </c>
-      <c r="H171" s="2" t="n"/>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="60" customHeight="1">
       <c r="A172" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add 52 A1.2 unit 6 frequency questions and suggested answers
</commit_message>
<xml_diff>
--- a/data/speakingcards_questions.xlsx
+++ b/data/speakingcards_questions.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speaking Cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Speaking Cards'!$A$1:$H$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Speaking Cards'!$A$1:$H$273</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8241,10 +8241,1882 @@
         </is>
       </c>
     </row>
+    <row r="222" ht="90" customHeight="1">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>How often do you exercise?</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr"/>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t>I usually exercise three times a week.</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="90" customHeight="1">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>How often do you eat breakfast?</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr"/>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t>I always eat breakfast in the morning.</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="90" customHeight="1">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>How often do you watch TV?</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr"/>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t>I usually watch TV in the evening.</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="90" customHeight="1">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>How often do you read books?</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr"/>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t>I often read books before bed.</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="226" ht="90" customHeight="1">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>How often do you go to the movies?</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr"/>
+      <c r="C226" s="2" t="inlineStr">
+        <is>
+          <t>I go to the movies once a month.</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E226" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F226" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G226" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H226" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="227" ht="90" customHeight="1">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>How often do you drink coffee?</t>
+        </is>
+      </c>
+      <c r="B227" s="2" t="inlineStr"/>
+      <c r="C227" s="2" t="inlineStr">
+        <is>
+          <t>I usually drink coffee every morning.</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E227" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F227" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G227" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H227" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="228" ht="90" customHeight="1">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>How often do you play video games?</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr"/>
+      <c r="C228" s="2" t="inlineStr">
+        <is>
+          <t>I sometimes play video games after class.</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E228" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G228" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H228" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="229" ht="90" customHeight="1">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>How often do you visit your family?</t>
+        </is>
+      </c>
+      <c r="B229" s="2" t="inlineStr"/>
+      <c r="C229" s="2" t="inlineStr">
+        <is>
+          <t>I visit my family twice a month.</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E229" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F229" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G229" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H229" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="230" ht="90" customHeight="1">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>How often do you study English?</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr"/>
+      <c r="C230" s="2" t="inlineStr">
+        <is>
+          <t>I always study English after dinner.</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E230" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F230" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G230" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H230" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="231" ht="90" customHeight="1">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>How often do you listen to music?</t>
+        </is>
+      </c>
+      <c r="B231" s="2" t="inlineStr"/>
+      <c r="C231" s="2" t="inlineStr">
+        <is>
+          <t>I listen to music every day.</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E231" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F231" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G231" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H231" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="232" ht="90" customHeight="1">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>How often do you eat fast food?</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr"/>
+      <c r="C232" s="2" t="inlineStr">
+        <is>
+          <t>I rarely eat fast food during the week.</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E232" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F232" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G232" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H232" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="233" ht="90" customHeight="1">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>How often do you cook dinner?</t>
+        </is>
+      </c>
+      <c r="B233" s="2" t="inlineStr"/>
+      <c r="C233" s="2" t="inlineStr">
+        <is>
+          <t>I usually cook dinner five times a week.</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E233" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F233" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G233" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H233" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="234" ht="90" customHeight="1">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>How often do you go shopping?</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr"/>
+      <c r="C234" s="2" t="inlineStr">
+        <is>
+          <t>I go shopping once a week.</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E234" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F234" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G234" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H234" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="235" ht="90" customHeight="1">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>How often do you clean your room?</t>
+        </is>
+      </c>
+      <c r="B235" s="2" t="inlineStr"/>
+      <c r="C235" s="2" t="inlineStr">
+        <is>
+          <t>I always clean my room on Saturdays.</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E235" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F235" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G235" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H235" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="236" ht="90" customHeight="1">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>How often do you go to bed late?</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr"/>
+      <c r="C236" s="2" t="inlineStr">
+        <is>
+          <t>I sometimes go to bed late on weekends.</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E236" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F236" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G236" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H236" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="237" ht="90" customHeight="1">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>How often do you walk to school or work?</t>
+        </is>
+      </c>
+      <c r="B237" s="2" t="inlineStr"/>
+      <c r="C237" s="2" t="inlineStr">
+        <is>
+          <t>I usually walk to school or work in the morning.</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E237" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F237" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G237" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H237" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="238" ht="90" customHeight="1">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>How often do you play sports?</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr"/>
+      <c r="C238" s="2" t="inlineStr">
+        <is>
+          <t>I play sports twice a week.</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E238" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F238" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G238" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H238" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="239" ht="90" customHeight="1">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>How often do you call your friends?</t>
+        </is>
+      </c>
+      <c r="B239" s="2" t="inlineStr"/>
+      <c r="C239" s="2" t="inlineStr">
+        <is>
+          <t>I often call my friends in the evening.</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E239" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F239" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G239" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H239" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="240" ht="90" customHeight="1">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>How often do you eat vegetables?</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr"/>
+      <c r="C240" s="2" t="inlineStr">
+        <is>
+          <t>I always eat vegetables at lunchtime.</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E240" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F240" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G240" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H240" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="241" ht="90" customHeight="1">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>How often do you travel?</t>
+        </is>
+      </c>
+      <c r="B241" s="2" t="inlineStr"/>
+      <c r="C241" s="2" t="inlineStr">
+        <is>
+          <t>I usually travel once a year.</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E241" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F241" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G241" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H241" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="242" ht="90" customHeight="1">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>How often do you take a bus?</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr"/>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>I take a bus every weekday.</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="243" ht="90" customHeight="1">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>How often do you go to the gym?</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr"/>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>I never go to the gym. I exercise at home every day.</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="244" ht="90" customHeight="1">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>How often do you do your homework?</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr"/>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>I always do my homework after class.</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="245" ht="90" customHeight="1">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>How often do you eat at a restaurant?</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr"/>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>I sometimes eat at a restaurant on Sundays.</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="246" ht="90" customHeight="1">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>How often do you use social media?</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr"/>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>I usually use social media twice a day.</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="247" ht="90" customHeight="1">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>How often do you go dancing?</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr"/>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>I hardly ever go dancing. I go once or twice a year.</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>How often, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="248" ht="90" customHeight="1">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Do you always eat breakfast?</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr"/>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I always eat breakfast before work.</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="249" ht="90" customHeight="1">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Do you always wake up early?</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr"/>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>No, I sometimes wake up late on Sundays.</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="250" ht="90" customHeight="1">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Do you always brush your teeth before bed?</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr"/>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I always brush my teeth before bed.</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E250" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="251" ht="90" customHeight="1">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Do you always study English after class?</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr"/>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>No, I usually study English in the evening.</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="252" ht="90" customHeight="1">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>Do you always walk to work or school?</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr"/>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>No, I sometimes take the bus.</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="90" customHeight="1">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Do you always drink coffee in the morning?</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr"/>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>No, I never drink coffee. I drink tea every morning.</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="254" ht="90" customHeight="1">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Do you always do your homework?</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr"/>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I always do my homework after dinner.</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="255" ht="90" customHeight="1">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Do you always cook dinner at home?</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr"/>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>No, I eat at a restaurant once a week.</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="256" ht="90" customHeight="1">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Do you always go to bed before ten?</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr"/>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>No, I sometimes go to bed at eleven.</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="257" ht="90" customHeight="1">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes watch movies at home?</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr"/>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I sometimes watch movies on Saturday nights.</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="258" ht="90" customHeight="1">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes play video games?</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr"/>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I play video games twice a week.</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="259" ht="90" customHeight="1">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes eat fast food?</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr"/>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I sometimes eat fast food on weekends.</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="260" ht="90" customHeight="1">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes visit your friends?</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr"/>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I usually visit my friends on Sundays.</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E260" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="261" ht="90" customHeight="1">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes listen to music while you study?</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr"/>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>No, I never listen to music while I study.</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="262" ht="90" customHeight="1">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes take a nap?</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr"/>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I sometimes take a nap after lunch.</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="263" ht="90" customHeight="1">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes go shopping after work?</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr"/>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I go shopping after work once a week.</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="264" ht="90" customHeight="1">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes forget your keys?</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr"/>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I sometimes forget my keys in the morning.</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="265" ht="90" customHeight="1">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>Do you sometimes cook for your family?</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr"/>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I usually cook for my family on Saturdays.</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="266" ht="90" customHeight="1">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently exercise?</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr"/>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I exercise four times a week.</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="267" ht="90" customHeight="1">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently use social media?</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr"/>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I use social media every day.</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="268" ht="90" customHeight="1">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently read books?</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr"/>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I usually read before bed.</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E268" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H268" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="90" customHeight="1">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently travel?</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr"/>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>No, I only travel once a year.</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="90" customHeight="1">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently call your family?</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr"/>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I call my family every evening.</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="271" ht="90" customHeight="1">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently go to the movies?</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr"/>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>No, I rarely go to the movies.</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
+    <row r="272" ht="90" customHeight="1">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently practice English with friends?</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr"/>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I practice English with friends three times a week.</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>Student A</t>
+        </is>
+      </c>
+    </row>
+    <row r="273" ht="90" customHeight="1">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>Do you frequently eat vegetables?</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr"/>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>Yes, I always eat vegetables with dinner.</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>Yes/No questions, Simple present, Adverbs of frequency, Time expressions</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>A1.2</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>Student B</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H221"/>
+  <autoFilter ref="A1:H273"/>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H221" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H221 H222:H273" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Student A,Student B"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add optional Spanish translations to cards and workbook
</commit_message>
<xml_diff>
--- a/data/speakingcards_questions.xlsx
+++ b/data/speakingcards_questions.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Speaking Cards" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Speaking Cards'!$A$1:$H$273</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Speaking Cards'!$A$1:$J$273</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H273"/>
+  <dimension ref="A1:J273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -441,6 +441,8 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,6 +486,16 @@
           <t>Student</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>QuestionTranslation</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>AnswerTranslation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -520,6 +532,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es Navidad?</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Navidad es el 25 de diciembre.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -556,6 +578,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es Año Nuevo?</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Es el 1 de enero.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -592,6 +624,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de San Valentín?</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Es el 14 de febrero.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -628,6 +670,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué mes es el Día Internacional de la Mujer?</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Es en marzo.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -664,6 +716,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo se celebra normalmente la Semana Santa?</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente se celebra en marzo o abril.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -700,6 +762,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Tierra?</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Es el 22 de abril.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -736,6 +808,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día del Trabajo?</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Es el 1 de mayo.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -772,6 +854,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Madre en Guatemala?</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Es el 10 de mayo.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -808,6 +900,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué mes es el Día del Padre?</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Es en junio.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -844,6 +946,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día del Maestro?</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Es el 25 de junio.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -880,6 +992,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día del Ejército?</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Es el 30 de junio.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -916,6 +1038,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Virgen de la Asunción?</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Es el 15 de agosto.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -952,6 +1084,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Bandera Nacional?</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Es el 17 de agosto.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -988,6 +1130,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Independencia?</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Es el 15 de septiembre.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1024,6 +1176,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué mes es el Día del Niño?</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Es en octubre.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1060,6 +1222,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Revolución?</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Es el 20 de octubre.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1096,6 +1268,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué mes es Halloween?</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Es en octubre.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1132,6 +1314,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de Todos los Santos?</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Es el 1 de noviembre.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1168,6 +1360,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es la Quema del Diablo?</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Es el 7 de diciembre.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1204,6 +1406,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es Navidad?</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Es el 25 de diciembre.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1240,6 +1452,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es la víspera de Año Nuevo?</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Es el 31 de diciembre.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1280,6 +1502,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es tu cumpleaños?</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Mi cumpleaños es el [Día] de [Mes].</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1320,6 +1552,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué mes es tu cumpleaños?</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Mi cumpleaños es en [Mes].</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1356,6 +1598,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos días tiene diciembre?</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Diciembre tiene 31 días.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1392,6 +1644,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos días tiene febrero?</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Febrero tiene 28 o 29 días.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1428,6 +1690,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos días tiene junio?</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Junio tiene 30 días.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1464,6 +1736,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo es el Día de la Independencia en Estados Unidos?</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Es el 4 de julio.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1504,6 +1786,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo naciste?</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Nací el [Día] de [Mes] de [Año].</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1544,6 +1836,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>¿En qué año naciste?</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Nací en [Año].</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -1580,6 +1882,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu día favorito de la semana?</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Mi día favorito es el viernes.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -1616,6 +1928,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu mes favorito del año?</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Mi mes favorito es diciembre.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -1656,6 +1978,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu estación favorita?</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Mi estación favorita es la temporada de lluvias.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -1692,6 +2024,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos hermanos tienes?</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Tengo dos hermanos.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1728,6 +2070,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas hermanas tienes?</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Tengo una hermana.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1764,6 +2116,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas mascotas tienes?</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Tengo una mascota.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1800,6 +2162,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde está tu casa?</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Mi casa está en la zona 1.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1836,6 +2208,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde está tu profesor o profesora?</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Está en el salón de clases.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1872,6 +2254,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde trabajas?</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Trabajo en una oficina.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1908,6 +2300,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde está tu mamá?</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Mi mamá está en casa.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1944,6 +2346,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>¿Estás feliz?</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Sí, estoy feliz. / No, no estoy feliz.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1980,6 +2392,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes hambre?</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tengo hambre. / No, no tengo hambre.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2016,6 +2438,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu mamá es de la ciudad de Guatemala?</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, no lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -2052,6 +2484,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>¿Estás casado o casada?</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo estoy. / No, no lo estoy.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -2088,6 +2530,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu mejor amistad es una mujer?</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Sí, es una mujer. / No, es un hombre.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -2124,6 +2576,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>¿Tus ojos son cafés?</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo son. / No, no lo son.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -2160,6 +2622,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes el cabello largo?</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo tengo largo. / No, no lo tengo largo.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2196,6 +2668,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu perro es amigable?</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, no lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -2232,6 +2714,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color es tu cabello?</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>Mi cabello es negro.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2268,6 +2760,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color son tus ojos?</t>
+        </is>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>Mis ojos son cafés.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2308,6 +2810,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color es el pelaje de tu mascota?</t>
+        </is>
+      </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>El pelaje de mi mascota es blanco.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2344,6 +2856,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>¿Estás en casa?</t>
+        </is>
+      </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>Sí, estoy en casa. / No, no estoy en casa.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2380,6 +2902,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu papá está en casa?</t>
+        </is>
+      </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>Sí, está en casa. / No, no está en casa.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -2416,6 +2948,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu mamá está en el trabajo?</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>Sí, está en el trabajo. / No, no está en el trabajo.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -2452,6 +2994,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>¿INTECAP está abierto en este momento?</t>
+        </is>
+      </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>Sí, está abierto. / No, no está abierto.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -2488,6 +3040,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>¿La clase es interesante?</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -2524,6 +3086,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo está tu mamá?</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>Está bien, gracias.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -2560,6 +3132,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo están tus padres?</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Están bien.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -2596,6 +3178,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo está tu profesora?</t>
+        </is>
+      </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>Está muy bien.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -2632,6 +3224,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>¿Estás soltero o soltera?</t>
+        </is>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo estoy. / No, no lo estoy.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -2668,6 +3270,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>¿Messi es de Argentina?</t>
+        </is>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -2704,6 +3316,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>¿Maradona es de Colombia?</t>
+        </is>
+      </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>No, no lo es. Es de Argentina.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -2740,6 +3362,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>¿Shakira es de Venezuela?</t>
+        </is>
+      </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>No, no lo es. Es de Colombia.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -2776,6 +3408,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>¿Los integrantes de BTS son de Japón?</t>
+        </is>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>No, no lo son. Son de Corea del Sur.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -2812,6 +3454,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>¿Arjona es un cantante de reggae?</t>
+        </is>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>No, no lo es. Es un cantante de pop.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -2848,6 +3500,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>¿Maná es una banda mexicana?</t>
+        </is>
+      </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -2884,6 +3546,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>¿Los tacos son una comida típica guatemalteca?</t>
+        </is>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>No, no lo son. Son mexicanos.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -2920,6 +3592,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>¿Los tamales son una comida típica guatemalteca?</t>
+        </is>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo son.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -2956,6 +3638,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde comes comida típica?</t>
+        </is>
+      </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>Como comida típica en el mercado.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -2992,6 +3684,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué lugares turísticos conoces?</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>Conozco Antigua y Tikal.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -3028,6 +3730,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu departamento favorito de Guatemala?</t>
+        </is>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Mi departamento favorito es Petén.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -3064,6 +3776,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I72" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos hermanos y sobrinos tienes?</t>
+        </is>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Tengo dos hermanos y tres sobrinos.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -3100,6 +3822,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I73" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas tías y tíos tienes?</t>
+        </is>
+      </c>
+      <c r="J73" s="2" t="inlineStr">
+        <is>
+          <t>Tengo cuatro tías y dos tíos.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -3136,6 +3868,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu tía favorita?</t>
+        </is>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>Mi tía favorita es María.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -3172,6 +3914,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I75" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes hermanos?</t>
+        </is>
+      </c>
+      <c r="J75" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tengo. / No, no tengo.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -3208,6 +3960,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I76" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes primos?</t>
+        </is>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tengo. / No, no tengo.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -3244,6 +4006,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I77" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos primos tienes?</t>
+        </is>
+      </c>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>Tengo diez primos.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -3280,6 +4052,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes sobrinas y sobrinos?</t>
+        </is>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tengo. / No, no tengo.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -3316,6 +4098,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I79" s="2" t="inlineStr">
+        <is>
+          <t>¿De dónde son tus padres?</t>
+        </is>
+      </c>
+      <c r="J79" s="2" t="inlineStr">
+        <is>
+          <t>Son de Guatemala.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -3352,6 +4144,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I80" s="2" t="inlineStr">
+        <is>
+          <t>¿De dónde es tu computadora?</t>
+        </is>
+      </c>
+      <c r="J80" s="2" t="inlineStr">
+        <is>
+          <t>Es de Estados Unidos.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -3388,6 +4190,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu abuela vive todavía?</t>
+        </is>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>Sí, vive. / No, ya no vive.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -3424,6 +4236,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu abuelo vive todavía?</t>
+        </is>
+      </c>
+      <c r="J82" s="2" t="inlineStr">
+        <is>
+          <t>Sí, vive. / No, ya no vive.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -3460,6 +4282,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I83" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu mamá?</t>
+        </is>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>Mi mamá es [Nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -3496,6 +4328,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu abuela materna?</t>
+        </is>
+      </c>
+      <c r="J84" s="2" t="inlineStr">
+        <is>
+          <t>Es [Nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -3532,6 +4374,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu abuela paterna?</t>
+        </is>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>Es [Nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -3568,6 +4420,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I86" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta tocar el piano?</t>
+        </is>
+      </c>
+      <c r="J86" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -3604,6 +4466,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I87" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta tocar algún instrumento?</t>
+        </is>
+      </c>
+      <c r="J87" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -3640,6 +4512,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I88" s="2" t="inlineStr">
+        <is>
+          <t>¿Prefieres la playa o las montañas?</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>Prefiero la playa.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -3676,6 +4558,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu animal favorito?</t>
+        </is>
+      </c>
+      <c r="J89" s="2" t="inlineStr">
+        <is>
+          <t>Mi animal favorito es el perro.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -3712,6 +4604,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué comida disfrutas comer?</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Disfruto comer pizza.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -3752,6 +4654,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I91" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué comida disfrutas cocinar?</t>
+        </is>
+      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>Disfruto cocinar pasta.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -3788,6 +4700,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué música te gusta escuchar?</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Me gusta escuchar música pop.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -3824,6 +4746,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu cantante favorito o favorita?</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>Mi cantante favorita es Dua Lipa.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -3860,6 +4792,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I94" s="2" t="inlineStr">
+        <is>
+          <t>¿Quién es tu deportista favorito o favorita?</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Mi jugador favorito es Messi.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -3896,6 +4838,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I95" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu deporte favorito?</t>
+        </is>
+      </c>
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>Mi deporte favorito es el fútbol.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -3932,6 +4884,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu materia favorita?</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>Mi materia favorita es inglés.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -3968,6 +4930,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu comida favorita?</t>
+        </is>
+      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>Mi comida favorita es el pollo.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -4008,6 +4980,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I98" s="2" t="inlineStr">
+        <is>
+          <t>¿La pasta es un platillo italiano?</t>
+        </is>
+      </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -4044,6 +5026,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I99" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu restaurante favorito?</t>
+        </is>
+      </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>Mi restaurante favorito es Pollo Campero.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -4080,6 +5072,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I100" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué país te gustaría visitar?</t>
+        </is>
+      </c>
+      <c r="J100" s="2" t="inlineStr">
+        <is>
+          <t>Me gustaría visitar Japón.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -4116,6 +5118,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I101" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo se deletrea Guatemala?</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>G-U-A-T-E-M-A-L-A.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -4152,6 +5164,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I102" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo se deletrea tu primer nombre?</t>
+        </is>
+      </c>
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>[Deletrea el nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -4188,6 +5210,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I103" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo se deletrea el nombre de tu profesor o profesora?</t>
+        </is>
+      </c>
+      <c r="J103" s="2" t="inlineStr">
+        <is>
+          <t>[Deletrea el nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -4224,6 +5256,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I104" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo se deletrea tu segundo nombre?</t>
+        </is>
+      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>[Deletrea el nombre].</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -4260,6 +5302,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I105" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo se deletrea tu apellido?</t>
+        </is>
+      </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>[Deletrea el apellido].</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -4296,6 +5348,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I106" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu comida guatemalteca favorita?</t>
+        </is>
+      </c>
+      <c r="J106" s="2" t="inlineStr">
+        <is>
+          <t>Mi comida guatemalteca favorita es el pepián.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -4332,6 +5394,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu dirección?</t>
+        </is>
+      </c>
+      <c r="J107" s="2" t="inlineStr">
+        <is>
+          <t>Mi dirección es 5.ª avenida, zona 4.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -4368,6 +5440,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I108" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu correo electrónico?</t>
+        </is>
+      </c>
+      <c r="J108" s="2" t="inlineStr">
+        <is>
+          <t>Mi correo electrónico es student@example.com.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -4404,6 +5486,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I109" s="2" t="inlineStr">
+        <is>
+          <t>¿Puedes deletrear en inglés el nombre de tu animal favorito?</t>
+        </is>
+      </c>
+      <c r="J109" s="2" t="inlineStr">
+        <is>
+          <t>D-O-G (perro).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -4440,6 +5532,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I110" s="2" t="inlineStr">
+        <is>
+          <t>¿Puedes deletrear en inglés el nombre de tu fruta favorita?</t>
+        </is>
+      </c>
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>A-P-P-L-E (manzana).</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -4476,6 +5578,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I111" s="2" t="inlineStr">
+        <is>
+          <t>¿Puedes deletrear en inglés el nombre de tu deporte favorito?</t>
+        </is>
+      </c>
+      <c r="J111" s="2" t="inlineStr">
+        <is>
+          <t>S-O-C-C-E-R (fútbol).</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -4512,6 +5624,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I112" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué películas te gusta ver?</t>
+        </is>
+      </c>
+      <c r="J112" s="2" t="inlineStr">
+        <is>
+          <t>Me gusta ver películas de acción.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -4548,6 +5670,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué libros te gusta leer?</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Me gusta leer novelas históricas.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -4584,6 +5716,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan las películas de ciencia ficción?</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustan. / No, no me gustan.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -4620,6 +5762,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I115" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan las películas románticas?</t>
+        </is>
+      </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustan. / No, no me gustan.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -4656,6 +5808,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I116" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan las películas de comedia?</t>
+        </is>
+      </c>
+      <c r="J116" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustan. / No, no me gustan.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -4692,6 +5854,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan las películas de acción?</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustan. / No, no me gustan.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -4728,6 +5900,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta ver anime?</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -4768,6 +5950,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I119" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta ver telenovelas?</t>
+        </is>
+      </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -4804,6 +5996,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta escribir?</t>
+        </is>
+      </c>
+      <c r="J120" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -4840,6 +6042,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I121" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta escuchar rock?</t>
+        </is>
+      </c>
+      <c r="J121" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -4876,6 +6088,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I122" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta escuchar música pop?</t>
+        </is>
+      </c>
+      <c r="J122" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -4912,6 +6134,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué pasatiempos tiene tu mamá?</t>
+        </is>
+      </c>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>Le gusta leer y cocinar.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -4948,6 +6180,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué pasatiempos tiene tu hermano o hermana?</t>
+        </is>
+      </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>A él le gusta jugar videojuegos.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -4984,6 +6226,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu casa tiene jardín?</t>
+        </is>
+      </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tiene. / No, no tiene.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -5020,6 +6272,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu casa tiene un patio delantero?</t>
+        </is>
+      </c>
+      <c r="J126" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tiene. / No, no tiene.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -5056,6 +6318,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I127" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu casa tiene un patio trasero?</t>
+        </is>
+      </c>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tiene. / No, no tiene.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -5092,6 +6364,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas habitaciones tiene tu casa?</t>
+        </is>
+      </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>Mi casa tiene tres habitaciones.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -5128,6 +6410,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas ventanas tiene tu habitación?</t>
+        </is>
+      </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>Mi habitación tiene dos ventanas.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -5164,6 +6456,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I130" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color es tu casa?</t>
+        </is>
+      </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>Mi casa es blanca.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -5200,6 +6502,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I131" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color es tu habitación?</t>
+        </is>
+      </c>
+      <c r="J131" s="2" t="inlineStr">
+        <is>
+          <t>Mi habitación es azul.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -5236,6 +6548,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I132" s="2" t="inlineStr">
+        <is>
+          <t>Menciona tres muebles que hay en tu habitación.</t>
+        </is>
+      </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>Hay una cama, un escritorio y una silla.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -5272,6 +6594,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I133" s="2" t="inlineStr">
+        <is>
+          <t>Menciona tres muebles que hay en tu sala.</t>
+        </is>
+      </c>
+      <c r="J133" s="2" t="inlineStr">
+        <is>
+          <t>Hay un sofá, un televisor y una mesa.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -5308,6 +6640,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I134" s="2" t="inlineStr">
+        <is>
+          <t>Menciona tres muebles que hay en tu cocina.</t>
+        </is>
+      </c>
+      <c r="J134" s="2" t="inlineStr">
+        <is>
+          <t>Hay una estufa, una refrigeradora y una mesa.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -5344,6 +6686,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu cocina tiene ventanas?</t>
+        </is>
+      </c>
+      <c r="J135" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tiene. / No, no tiene.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -5380,6 +6732,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I136" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu cocina tiene plantas?</t>
+        </is>
+      </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>Sí, tiene. / No, no tiene.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -5416,6 +6778,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I137" s="2" t="inlineStr">
+        <is>
+          <t>¿De qué color es la puerta de tu dormitorio?</t>
+        </is>
+      </c>
+      <c r="J137" s="2" t="inlineStr">
+        <is>
+          <t>Es café.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -5452,6 +6824,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I138" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría ir al museo? ¿A cuál?</t>
+        </is>
+      </c>
+      <c r="J138" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. Quiero ir al Museo Miraflores.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -5488,6 +6870,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I139" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría ir al zoológico? ¿Qué animal te gustaría observar?</t>
+        </is>
+      </c>
+      <c r="J139" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. Quiero observar a los monos.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -5524,6 +6916,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I140" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría ir a la biblioteca? ¿Qué libro te gustaría leer?</t>
+        </is>
+      </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. Quiero leer una novela.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -5560,6 +6962,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I141" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría ir a la librería? ¿Qué libro te gustaría comprar?</t>
+        </is>
+      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. Quiero comprar un diccionario.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -5596,6 +7008,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I142" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría ir al centro comercial? ¿A cuál te gustaría ir?</t>
+        </is>
+      </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. Quiero ir a Miraflores.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -5632,6 +7054,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I143" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué días compras los alimentos?</t>
+        </is>
+      </c>
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>Compro los alimentos los sábados.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -5668,6 +7100,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I144" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué días estudias inglés?</t>
+        </is>
+      </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>Estudio inglés los martes y los jueves.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -5704,6 +7146,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I145" s="2" t="inlineStr">
+        <is>
+          <t>¿A qué hora haces la tarea?</t>
+        </is>
+      </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>Hago la tarea a las siete de la noche.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -5740,6 +7192,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I146" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre desayunas?</t>
+        </is>
+      </c>
+      <c r="J146" s="2" t="inlineStr">
+        <is>
+          <t>Sí, siempre desayuno. / No, a veces no desayuno.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -5776,6 +7238,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I147" s="2" t="inlineStr">
+        <is>
+          <t>¿Normalmente cenas?</t>
+        </is>
+      </c>
+      <c r="J147" s="2" t="inlineStr">
+        <is>
+          <t>Sí, normalmente ceno.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -5812,6 +7284,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I148" s="2" t="inlineStr">
+        <is>
+          <t>¿Con quién cenas?</t>
+        </is>
+      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>Ceno con mi familia.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -5848,6 +7330,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I149" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde desayunas normalmente?</t>
+        </is>
+      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente desayuno en la cocina.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -5884,6 +7376,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I150" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde almuerzas normalmente?</t>
+        </is>
+      </c>
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente almuerzo en el trabajo.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -5920,6 +7422,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I151" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas personas viven en tu casa?</t>
+        </is>
+      </c>
+      <c r="J151" s="2" t="inlineStr">
+        <is>
+          <t>Cuatro personas viven en mi casa.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -5956,6 +7468,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I152" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu festividad favorita?</t>
+        </is>
+      </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>Mi festividad favorita es Navidad.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -5992,6 +7514,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I153" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta celebrar Halloween?</t>
+        </is>
+      </c>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -6028,6 +7560,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I154" s="2" t="inlineStr">
+        <is>
+          <t>¿Normalmente celebras Halloween?</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo celebro. / No, no lo celebro.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -6064,6 +7606,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I155" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta celebrar Navidad?</t>
+        </is>
+      </c>
+      <c r="J155" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gusta. / No, no me gusta.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -6100,6 +7652,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I156" s="2" t="inlineStr">
+        <is>
+          <t>¿Normalmente celebras tu cumpleaños?</t>
+        </is>
+      </c>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo celebro. / No, no lo celebro.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -6136,6 +7698,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I157" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde celebras tu cumpleaños?</t>
+        </is>
+      </c>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>Lo celebro en un restaurante o en casa.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -6172,6 +7744,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I158" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu casa es grande?</t>
+        </is>
+      </c>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, es pequeña.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -6208,6 +7790,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I159" s="2" t="inlineStr">
+        <is>
+          <t>¿Los perros son tus mascotas favoritas?</t>
+        </is>
+      </c>
+      <c r="J159" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo son. / No, no lo son.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -6244,6 +7836,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>¿Los gatos son tus animales favoritos?</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo son. / No, no lo son.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -6280,6 +7882,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I161" s="2" t="inlineStr">
+        <is>
+          <t>¿El inglés es fácil para ti?</t>
+        </is>
+      </c>
+      <c r="J161" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, es difícil.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -6316,6 +7928,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I162" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde vives?</t>
+        </is>
+      </c>
+      <c r="J162" s="2" t="inlineStr">
+        <is>
+          <t>Vivo en la ciudad de Guatemala.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -6352,6 +7974,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>¿Vives en la ciudad o en el campo?</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>Vivo en la ciudad.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -6388,6 +8020,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I164" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu mamá es maestra?</t>
+        </is>
+      </c>
+      <c r="J164" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, no lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -6424,6 +8066,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>¿Eres arquitecto o arquitecta?</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo soy. / No, soy docente.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -6460,6 +8112,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>¿Tu papá es médico?</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo es. / No, no lo es.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -6496,6 +8158,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>¿Tus hermanos son ingenieros?</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>Sí, lo son. / No, no lo son.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -6532,6 +8204,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I168" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué trabajo te gustaría tener?</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>Me gustaría ser gerente.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -6568,6 +8250,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustaría vivir en la ciudad?</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>Sí, me gustaría. / No, prefiero el campo.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -6604,6 +8296,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué música odias escuchar?</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>Odio escuchar heavy metal.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -6638,6 +8340,16 @@
       <c r="H171" s="2" t="inlineStr">
         <is>
           <t>Student B</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuál es tu color favorito?</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>Mi color favorito es el azul.</t>
         </is>
       </c>
     </row>
@@ -6672,6 +8384,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I172" s="2" t="inlineStr">
+        <is>
+          <t>¿Juegas videojuegos?</t>
+        </is>
+      </c>
+      <c r="J172" s="2" t="inlineStr"/>
     </row>
     <row r="173" ht="60" customHeight="1">
       <c r="A173" s="2" t="inlineStr">
@@ -6704,6 +8422,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>¿Lees libros en tu tiempo libre?</t>
+        </is>
+      </c>
+      <c r="J173" s="2" t="inlineStr"/>
     </row>
     <row r="174" ht="60" customHeight="1">
       <c r="A174" s="2" t="inlineStr">
@@ -6736,6 +8460,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué tipo de música escuchas?</t>
+        </is>
+      </c>
+      <c r="J174" s="2" t="inlineStr"/>
     </row>
     <row r="175" ht="60" customHeight="1">
       <c r="A175" s="2" t="inlineStr">
@@ -6768,6 +8498,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>¿Tocas algún instrumento musical?</t>
+        </is>
+      </c>
+      <c r="J175" s="2" t="inlineStr"/>
     </row>
     <row r="176" ht="60" customHeight="1">
       <c r="A176" s="2" t="inlineStr">
@@ -6800,6 +8536,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué haces los fines de semana?</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr"/>
     </row>
     <row r="177" ht="60" customHeight="1">
       <c r="A177" s="2" t="inlineStr">
@@ -6832,6 +8574,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>¿Ves series en Netflix?</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr"/>
     </row>
     <row r="178" ht="60" customHeight="1">
       <c r="A178" s="2" t="inlineStr">
@@ -6864,6 +8612,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué tipo de películas te gustan?</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr"/>
     </row>
     <row r="179" ht="60" customHeight="1">
       <c r="A179" s="2" t="inlineStr">
@@ -6896,6 +8650,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan los deportes?</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr"/>
     </row>
     <row r="180" ht="60" customHeight="1">
       <c r="A180" s="2" t="inlineStr">
@@ -6928,6 +8688,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué deporte practicas?</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr"/>
     </row>
     <row r="181" ht="60" customHeight="1">
       <c r="A181" s="2" t="inlineStr">
@@ -6960,6 +8726,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>¿Vas al gimnasio?</t>
+        </is>
+      </c>
+      <c r="J181" s="2" t="inlineStr"/>
     </row>
     <row r="182" ht="60" customHeight="1">
       <c r="A182" s="2" t="inlineStr">
@@ -6992,6 +8764,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>¿A qué hora te despiertas?</t>
+        </is>
+      </c>
+      <c r="J182" s="2" t="inlineStr"/>
     </row>
     <row r="183" ht="60" customHeight="1">
       <c r="A183" s="2" t="inlineStr">
@@ -7024,6 +8802,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>¿Tomas café por la mañana?</t>
+        </is>
+      </c>
+      <c r="J183" s="2" t="inlineStr"/>
     </row>
     <row r="184" ht="60" customHeight="1">
       <c r="A184" s="2" t="inlineStr">
@@ -7056,6 +8840,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I184" s="2" t="inlineStr">
+        <is>
+          <t>¿Desayunas todos los días?</t>
+        </is>
+      </c>
+      <c r="J184" s="2" t="inlineStr"/>
     </row>
     <row r="185" ht="60" customHeight="1">
       <c r="A185" s="2" t="inlineStr">
@@ -7088,6 +8878,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I185" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué desayunas?</t>
+        </is>
+      </c>
+      <c r="J185" s="2" t="inlineStr"/>
     </row>
     <row r="186" ht="60" customHeight="1">
       <c r="A186" s="2" t="inlineStr">
@@ -7120,6 +8916,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>¿Cómo te trasladas al trabajo o a tu lugar de estudio?</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr"/>
     </row>
     <row r="187" ht="60" customHeight="1">
       <c r="A187" s="2" t="inlineStr">
@@ -7152,6 +8954,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>¿Conduces un carro?</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr"/>
     </row>
     <row r="188" ht="60" customHeight="1">
       <c r="A188" s="2" t="inlineStr">
@@ -7184,6 +8992,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I188" s="2" t="inlineStr">
+        <is>
+          <t>¿A qué hora terminas tu día?</t>
+        </is>
+      </c>
+      <c r="J188" s="2" t="inlineStr"/>
     </row>
     <row r="189" ht="60" customHeight="1">
       <c r="A189" s="2" t="inlineStr">
@@ -7216,6 +9030,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>¿Preparas tus propias comidas?</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr"/>
     </row>
     <row r="190" ht="60" customHeight="1">
       <c r="A190" s="2" t="inlineStr">
@@ -7248,6 +9068,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuándo estudias inglés?</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr"/>
     </row>
     <row r="191" ht="60" customHeight="1">
       <c r="A191" s="2" t="inlineStr">
@@ -7280,6 +9106,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>¿Duermes ocho horas al día?</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr"/>
     </row>
     <row r="192" ht="60" customHeight="1">
       <c r="A192" s="2" t="inlineStr">
@@ -7312,6 +9144,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta la comida picante?</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr"/>
     </row>
     <row r="193" ht="60" customHeight="1">
       <c r="A193" s="2" t="inlineStr">
@@ -7344,6 +9182,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I193" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué comida te gusta más?</t>
+        </is>
+      </c>
+      <c r="J193" s="2" t="inlineStr"/>
     </row>
     <row r="194" ht="60" customHeight="1">
       <c r="A194" s="2" t="inlineStr">
@@ -7376,6 +9220,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I194" s="2" t="inlineStr">
+        <is>
+          <t>¿Prefieres té o café?</t>
+        </is>
+      </c>
+      <c r="J194" s="2" t="inlineStr"/>
     </row>
     <row r="195" ht="60" customHeight="1">
       <c r="A195" s="2" t="inlineStr">
@@ -7408,6 +9258,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I195" s="2" t="inlineStr">
+        <is>
+          <t>¿Comes comida rápida?</t>
+        </is>
+      </c>
+      <c r="J195" s="2" t="inlineStr"/>
     </row>
     <row r="196" ht="60" customHeight="1">
       <c r="A196" s="2" t="inlineStr">
@@ -7440,6 +9296,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I196" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué tomas en las fiestas?</t>
+        </is>
+      </c>
+      <c r="J196" s="2" t="inlineStr"/>
     </row>
     <row r="197" ht="60" customHeight="1">
       <c r="A197" s="2" t="inlineStr">
@@ -7472,6 +9334,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t>¿Disfrutas cocinar?</t>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr"/>
     </row>
     <row r="198" ht="60" customHeight="1">
       <c r="A198" s="2" t="inlineStr">
@@ -7504,6 +9372,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gustan las verduras?</t>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr"/>
     </row>
     <row r="199" ht="60" customHeight="1">
       <c r="A199" s="2" t="inlineStr">
@@ -7536,6 +9410,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué postre te encanta?</t>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr"/>
     </row>
     <row r="200" ht="60" customHeight="1">
       <c r="A200" s="2" t="inlineStr">
@@ -7568,6 +9448,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>¿Comes carne?</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr"/>
     </row>
     <row r="201" ht="60" customHeight="1">
       <c r="A201" s="2" t="inlineStr">
@@ -7600,6 +9486,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>¿Pides comida por internet?</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr"/>
     </row>
     <row r="202" ht="60" customHeight="1">
       <c r="A202" s="2" t="inlineStr">
@@ -7632,6 +9524,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>¿Dónde trabajas?</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr"/>
     </row>
     <row r="203" ht="60" customHeight="1">
       <c r="A203" s="2" t="inlineStr">
@@ -7664,6 +9562,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>¿Te gusta tu trabajo?</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr"/>
     </row>
     <row r="204" ht="60" customHeight="1">
       <c r="A204" s="2" t="inlineStr">
@@ -7696,6 +9600,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué estudias?</t>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr"/>
     </row>
     <row r="205" ht="60" customHeight="1">
       <c r="A205" s="2" t="inlineStr">
@@ -7728,6 +9638,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t>¿Usas una computadora todos los días?</t>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr"/>
     </row>
     <row r="206" ht="60" customHeight="1">
       <c r="A206" s="2" t="inlineStr">
@@ -7760,6 +9676,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántas horas trabajas?</t>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr"/>
     </row>
     <row r="207" ht="60" customHeight="1">
       <c r="A207" s="2" t="inlineStr">
@@ -7792,6 +9714,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t>¿Trabajas desde casa?</t>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr"/>
     </row>
     <row r="208" ht="60" customHeight="1">
       <c r="A208" s="2" t="inlineStr">
@@ -7824,6 +9752,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t>¿Quieres aprender otro idioma?</t>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr"/>
     </row>
     <row r="209" ht="60" customHeight="1">
       <c r="A209" s="2" t="inlineStr">
@@ -7856,6 +9790,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t>¿Por qué estudias inglés?</t>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr"/>
     </row>
     <row r="210" ht="60" customHeight="1">
       <c r="A210" s="2" t="inlineStr">
@@ -7888,6 +9828,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>¿Lees las noticias?</t>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr"/>
     </row>
     <row r="211" ht="60" customHeight="1">
       <c r="A211" s="2" t="inlineStr">
@@ -7920,6 +9866,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>¿Ayudas a tus compañeros de clase?</t>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr"/>
     </row>
     <row r="212" ht="60" customHeight="1">
       <c r="A212" s="2" t="inlineStr">
@@ -7952,6 +9904,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>¿Tienes mascotas?</t>
+        </is>
+      </c>
+      <c r="J212" s="2" t="inlineStr"/>
     </row>
     <row r="213" ht="60" customHeight="1">
       <c r="A213" s="2" t="inlineStr">
@@ -7984,6 +9942,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>¿Qué animal te gusta?</t>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr"/>
     </row>
     <row r="214" ht="60" customHeight="1">
       <c r="A214" s="2" t="inlineStr">
@@ -8016,6 +9980,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>¿Vives con tu familia?</t>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr"/>
     </row>
     <row r="215" ht="60" customHeight="1">
       <c r="A215" s="2" t="inlineStr">
@@ -8048,6 +10018,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>¿Cuántos hermanos tienes?</t>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr"/>
     </row>
     <row r="216" ht="60" customHeight="1">
       <c r="A216" s="2" t="inlineStr">
@@ -8080,6 +10056,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>¿Viajas mucho?</t>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr"/>
     </row>
     <row r="217" ht="60" customHeight="1">
       <c r="A217" s="2" t="inlineStr">
@@ -8112,6 +10094,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>¿A dónde quieres viajar?</t>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr"/>
     </row>
     <row r="218" ht="60" customHeight="1">
       <c r="A218" s="2" t="inlineStr">
@@ -8144,6 +10132,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>¿Hablas otro idioma?</t>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr"/>
     </row>
     <row r="219" ht="60" customHeight="1">
       <c r="A219" s="2" t="inlineStr">
@@ -8176,6 +10170,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t>¿Coleccionas algo?</t>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr"/>
     </row>
     <row r="220" ht="60" customHeight="1">
       <c r="A220" s="2" t="inlineStr">
@@ -8208,6 +10208,12 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t>¿Sales con amigos los viernes?</t>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr"/>
     </row>
     <row r="221" ht="60" customHeight="1">
       <c r="A221" s="2" t="inlineStr">
@@ -8240,6 +10246,12 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>¿Juegas juegos de mesa?</t>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr"/>
     </row>
     <row r="222" ht="90" customHeight="1">
       <c r="A222" s="2" t="inlineStr">
@@ -8276,6 +10288,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia haces ejercicio?</t>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente hago ejercicio tres veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="90" customHeight="1">
       <c r="A223" s="2" t="inlineStr">
@@ -8312,6 +10334,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia desayunas?</t>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t>Siempre desayuno por la mañana.</t>
+        </is>
+      </c>
     </row>
     <row r="224" ht="90" customHeight="1">
       <c r="A224" s="2" t="inlineStr">
@@ -8348,6 +10380,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia ves televisión?</t>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente veo televisión por la noche.</t>
+        </is>
+      </c>
     </row>
     <row r="225" ht="90" customHeight="1">
       <c r="A225" s="2" t="inlineStr">
@@ -8384,6 +10426,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia lees libros?</t>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>A menudo leo libros antes de acostarme.</t>
+        </is>
+      </c>
     </row>
     <row r="226" ht="90" customHeight="1">
       <c r="A226" s="2" t="inlineStr">
@@ -8420,6 +10472,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I226" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia vas al cine?</t>
+        </is>
+      </c>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>Voy al cine una vez al mes.</t>
+        </is>
+      </c>
     </row>
     <row r="227" ht="90" customHeight="1">
       <c r="A227" s="2" t="inlineStr">
@@ -8456,6 +10518,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia tomas café?</t>
+        </is>
+      </c>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente tomo café todas las mañanas.</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="90" customHeight="1">
       <c r="A228" s="2" t="inlineStr">
@@ -8492,6 +10564,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I228" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia juegas videojuegos?</t>
+        </is>
+      </c>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>A veces juego videojuegos después de clase.</t>
+        </is>
+      </c>
     </row>
     <row r="229" ht="90" customHeight="1">
       <c r="A229" s="2" t="inlineStr">
@@ -8528,6 +10610,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I229" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia visitas a tu familia?</t>
+        </is>
+      </c>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>Visito a mi familia dos veces al mes.</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="90" customHeight="1">
       <c r="A230" s="2" t="inlineStr">
@@ -8564,6 +10656,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia estudias inglés?</t>
+        </is>
+      </c>
+      <c r="J230" s="2" t="inlineStr">
+        <is>
+          <t>Siempre estudio inglés después de cenar.</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="90" customHeight="1">
       <c r="A231" s="2" t="inlineStr">
@@ -8600,6 +10702,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I231" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia escuchas música?</t>
+        </is>
+      </c>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>Escucho música todos los días.</t>
+        </is>
+      </c>
     </row>
     <row r="232" ht="90" customHeight="1">
       <c r="A232" s="2" t="inlineStr">
@@ -8636,6 +10748,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I232" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia comes comida rápida?</t>
+        </is>
+      </c>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>Rara vez como comida rápida durante la semana.</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="90" customHeight="1">
       <c r="A233" s="2" t="inlineStr">
@@ -8672,6 +10794,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I233" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia preparas la cena?</t>
+        </is>
+      </c>
+      <c r="J233" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente preparo la cena cinco veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="234" ht="90" customHeight="1">
       <c r="A234" s="2" t="inlineStr">
@@ -8708,6 +10840,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia vas de compras?</t>
+        </is>
+      </c>
+      <c r="J234" s="2" t="inlineStr">
+        <is>
+          <t>Voy de compras una vez por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="235" ht="90" customHeight="1">
       <c r="A235" s="2" t="inlineStr">
@@ -8744,6 +10886,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia limpias tu habitación?</t>
+        </is>
+      </c>
+      <c r="J235" s="2" t="inlineStr">
+        <is>
+          <t>Siempre limpio mi habitación los sábados.</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="90" customHeight="1">
       <c r="A236" s="2" t="inlineStr">
@@ -8780,6 +10932,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia te acuestas tarde?</t>
+        </is>
+      </c>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>A veces me acuesto tarde los fines de semana.</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="90" customHeight="1">
       <c r="A237" s="2" t="inlineStr">
@@ -8816,6 +10978,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia vas caminando a la escuela o al trabajo?</t>
+        </is>
+      </c>
+      <c r="J237" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente voy caminando a la escuela o al trabajo por la mañana.</t>
+        </is>
+      </c>
     </row>
     <row r="238" ht="90" customHeight="1">
       <c r="A238" s="2" t="inlineStr">
@@ -8852,6 +11024,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I238" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia practicas deportes?</t>
+        </is>
+      </c>
+      <c r="J238" s="2" t="inlineStr">
+        <is>
+          <t>Practico deportes dos veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="90" customHeight="1">
       <c r="A239" s="2" t="inlineStr">
@@ -8888,6 +11070,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia llamas a tus amigos?</t>
+        </is>
+      </c>
+      <c r="J239" s="2" t="inlineStr">
+        <is>
+          <t>A menudo llamo a mis amigos por la noche.</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="90" customHeight="1">
       <c r="A240" s="2" t="inlineStr">
@@ -8924,6 +11116,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia comes verduras?</t>
+        </is>
+      </c>
+      <c r="J240" s="2" t="inlineStr">
+        <is>
+          <t>Siempre como verduras a la hora del almuerzo.</t>
+        </is>
+      </c>
     </row>
     <row r="241" ht="90" customHeight="1">
       <c r="A241" s="2" t="inlineStr">
@@ -8960,6 +11162,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I241" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia viajas?</t>
+        </is>
+      </c>
+      <c r="J241" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente viajo una vez al año.</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="90" customHeight="1">
       <c r="A242" s="2" t="inlineStr">
@@ -8996,6 +11208,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia tomas un bus?</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>Tomo un bus de lunes a viernes.</t>
+        </is>
+      </c>
     </row>
     <row r="243" ht="90" customHeight="1">
       <c r="A243" s="2" t="inlineStr">
@@ -9032,6 +11254,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia vas al gimnasio?</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>Nunca voy al gimnasio. Hago ejercicio en casa todos los días.</t>
+        </is>
+      </c>
     </row>
     <row r="244" ht="90" customHeight="1">
       <c r="A244" s="2" t="inlineStr">
@@ -9068,6 +11300,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia haces la tarea?</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>Siempre hago la tarea después de clase.</t>
+        </is>
+      </c>
     </row>
     <row r="245" ht="90" customHeight="1">
       <c r="A245" s="2" t="inlineStr">
@@ -9104,6 +11346,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia comes en un restaurante?</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>A veces como en un restaurante los domingos.</t>
+        </is>
+      </c>
     </row>
     <row r="246" ht="90" customHeight="1">
       <c r="A246" s="2" t="inlineStr">
@@ -9140,6 +11392,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia usas las redes sociales?</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>Normalmente uso las redes sociales dos veces al día.</t>
+        </is>
+      </c>
     </row>
     <row r="247" ht="90" customHeight="1">
       <c r="A247" s="2" t="inlineStr">
@@ -9176,6 +11438,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>¿Con qué frecuencia sales a bailar?</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>Casi nunca salgo a bailar. Voy una o dos veces al año.</t>
+        </is>
+      </c>
     </row>
     <row r="248" ht="90" customHeight="1">
       <c r="A248" s="2" t="inlineStr">
@@ -9212,6 +11484,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre desayunas?</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>Sí, siempre desayuno antes de trabajar.</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="90" customHeight="1">
       <c r="A249" s="2" t="inlineStr">
@@ -9248,6 +11530,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre te despiertas temprano?</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>No, a veces me despierto tarde los domingos.</t>
+        </is>
+      </c>
     </row>
     <row r="250" ht="90" customHeight="1">
       <c r="A250" s="2" t="inlineStr">
@@ -9284,6 +11576,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre te cepillas los dientes antes de acostarte?</t>
+        </is>
+      </c>
+      <c r="J250" s="2" t="inlineStr">
+        <is>
+          <t>Sí, siempre me cepillo los dientes antes de acostarme.</t>
+        </is>
+      </c>
     </row>
     <row r="251" ht="90" customHeight="1">
       <c r="A251" s="2" t="inlineStr">
@@ -9320,6 +11622,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre estudias inglés después de clase?</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>No, normalmente estudio inglés por la noche.</t>
+        </is>
+      </c>
     </row>
     <row r="252" ht="90" customHeight="1">
       <c r="A252" s="2" t="inlineStr">
@@ -9356,6 +11668,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre vas caminando al trabajo o a la escuela?</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>No, a veces tomo el bus.</t>
+        </is>
+      </c>
     </row>
     <row r="253" ht="90" customHeight="1">
       <c r="A253" s="2" t="inlineStr">
@@ -9392,6 +11714,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre tomas café por la mañana?</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>No, nunca tomo café. Tomo té todas las mañanas.</t>
+        </is>
+      </c>
     </row>
     <row r="254" ht="90" customHeight="1">
       <c r="A254" s="2" t="inlineStr">
@@ -9428,6 +11760,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre haces la tarea?</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>Sí, siempre hago la tarea después de cenar.</t>
+        </is>
+      </c>
     </row>
     <row r="255" ht="90" customHeight="1">
       <c r="A255" s="2" t="inlineStr">
@@ -9464,6 +11806,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre preparas la cena en casa?</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>No, como en un restaurante una vez por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="90" customHeight="1">
       <c r="A256" s="2" t="inlineStr">
@@ -9500,6 +11852,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>¿Siempre te acuestas antes de las diez?</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>No, a veces me acuesto a las once.</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="90" customHeight="1">
       <c r="A257" s="2" t="inlineStr">
@@ -9536,6 +11898,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces ves películas en casa?</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>Sí, a veces veo películas los sábados por la noche.</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="90" customHeight="1">
       <c r="A258" s="2" t="inlineStr">
@@ -9572,6 +11944,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces juegas videojuegos?</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>Sí, juego videojuegos dos veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="90" customHeight="1">
       <c r="A259" s="2" t="inlineStr">
@@ -9608,6 +11990,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces comes comida rápida?</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>Sí, a veces como comida rápida los fines de semana.</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="90" customHeight="1">
       <c r="A260" s="2" t="inlineStr">
@@ -9644,6 +12036,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces visitas a tus amigos?</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>Sí, normalmente visito a mis amigos los domingos.</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="90" customHeight="1">
       <c r="A261" s="2" t="inlineStr">
@@ -9680,6 +12082,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces escuchas música mientras estudias?</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>No, nunca escucho música mientras estudio.</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="90" customHeight="1">
       <c r="A262" s="2" t="inlineStr">
@@ -9716,6 +12128,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces tomas una siesta?</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>Sí, a veces tomo una siesta después de almorzar.</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="90" customHeight="1">
       <c r="A263" s="2" t="inlineStr">
@@ -9752,6 +12174,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces vas de compras después del trabajo?</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>Sí, voy de compras después del trabajo una vez por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="90" customHeight="1">
       <c r="A264" s="2" t="inlineStr">
@@ -9788,6 +12220,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces olvidas tus llaves?</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>Sí, a veces olvido mis llaves por la mañana.</t>
+        </is>
+      </c>
     </row>
     <row r="265" ht="90" customHeight="1">
       <c r="A265" s="2" t="inlineStr">
@@ -9824,6 +12266,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I265" s="2" t="inlineStr">
+        <is>
+          <t>¿A veces cocinas para tu familia?</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>Sí, normalmente cocino para mi familia los sábados.</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="90" customHeight="1">
       <c r="A266" s="2" t="inlineStr">
@@ -9860,6 +12312,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>¿Haces ejercicio frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>Sí, hago ejercicio cuatro veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="267" ht="90" customHeight="1">
       <c r="A267" s="2" t="inlineStr">
@@ -9896,6 +12358,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>¿Usas las redes sociales frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>Sí, uso las redes sociales todos los días.</t>
+        </is>
+      </c>
     </row>
     <row r="268" ht="90" customHeight="1">
       <c r="A268" s="2" t="inlineStr">
@@ -9932,6 +12404,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I268" s="2" t="inlineStr">
+        <is>
+          <t>¿Lees libros frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J268" s="2" t="inlineStr">
+        <is>
+          <t>Sí, normalmente leo antes de acostarme.</t>
+        </is>
+      </c>
     </row>
     <row r="269" ht="90" customHeight="1">
       <c r="A269" s="2" t="inlineStr">
@@ -9968,6 +12450,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I269" s="2" t="inlineStr">
+        <is>
+          <t>¿Viajas frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>No, solo viajo una vez al año.</t>
+        </is>
+      </c>
     </row>
     <row r="270" ht="90" customHeight="1">
       <c r="A270" s="2" t="inlineStr">
@@ -10004,6 +12496,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t>¿Llamas a tu familia frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>Sí, llamo a mi familia todas las noches.</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="90" customHeight="1">
       <c r="A271" s="2" t="inlineStr">
@@ -10040,6 +12542,16 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>¿Vas al cine frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>No, rara vez voy al cine.</t>
+        </is>
+      </c>
     </row>
     <row r="272" ht="90" customHeight="1">
       <c r="A272" s="2" t="inlineStr">
@@ -10076,6 +12588,16 @@
           <t>Student A</t>
         </is>
       </c>
+      <c r="I272" s="2" t="inlineStr">
+        <is>
+          <t>¿Practicas inglés con amigos frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>Sí, practico inglés con amigos tres veces por semana.</t>
+        </is>
+      </c>
     </row>
     <row r="273" ht="90" customHeight="1">
       <c r="A273" s="2" t="inlineStr">
@@ -10112,9 +12634,19 @@
           <t>Student B</t>
         </is>
       </c>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>¿Comes verduras frecuentemente?</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>Sí, siempre como verduras con la cena.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H273"/>
+  <autoFilter ref="A1:J273"/>
   <dataValidations count="1">
     <dataValidation sqref="H2:H221 H222:H273" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Student A,Student B"</formula1>

</xml_diff>